<commit_message>
Apply user decisions on the 5 ambiguous new-products matches
59, 3051, and cervical collar set to explicit NA (0 units 2026) per
user instruction - none of the candidate matches found were correct.
MSG001F 0 merged across all 3 color variants (MSG001FB/FC/FW) into a
single row: 46 units / ₪37,922.88 across 4 channels. Orange
ambiguity table removed - all 5 cases now in the main table with
final values and a note documenting these are explicit user
decisions, not automatic merges.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QvuhBZminJvrtKVH8YY8
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-09-25-new-products-match.xlsx
+++ b/kirill/outputs/2026-09-25-new-products-match.xlsx
@@ -72,15 +72,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="79">
-  <si>
-    <t xml:space="preserve">מוצרים חדשים - התאמת כמות/כסף 2026 בפועל (YTD) לפי ערוץ מכירה - גרסה מתוקנת (סריקה מלאה על כל 34 מקורות)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="77">
+  <si>
+    <t xml:space="preserve">מוצרים חדשים - התאמת כמות/כסף 2026 בפועל (YTD) לפי ערוץ מכירה - גרסה סופית (כל 5 אי-הוודאויות הוכרעו ע"י המשתמש)</t>
   </si>
   <si>
     <t xml:space="preserve">תאריך חישוב:</t>
   </si>
   <si>
-    <t xml:space="preserve">תיקון (25/09/2026): בגרסה הקודמת נעשה שימוש בקוד CHEMIPAL המספרי (כמו 4411030) כמפתח חיפוש עבור דגמים שהותאמו דרך TRANS/הקטלוג (213 CTS, SH422, 397A, SH333) - זה תפס נכון מול 5 גיליונות CEMIUP0.9 (שם עמודת הקוד היא באמת הקוד המספרי), אבל פספס לגמרי את 29 גיליונות ה-SALES הישירים (שם עמודת "Product Code" מכילה את הקוד הטקסטואלי הגולמי כמו "213CTSR L", לא את הקוד המספרי) - בעיית אי-התאמת סוג-מפתח, לא בדיוק בעיית רווחים כפי שהועלתה. התיקון: סריקה חדשה לגמרי שמחפשת את קידומת-הבסיס הטקסטואלית (עם נרמול רווחים/מקפים/פלוס) ישירות מול עמודת הקוד הגולמית + שם המוצר בכל 34 המקורות (5 CEMIUP0.9 + 29 SALES, ללא 107/113 שכבר כלולות בתוך בתי מרקחת/מאוחדת - מניעת כפל ספירה). כמות/כסף = 2026 בפועל עד היום (YTD), לא מנורמל. כאשר דגם כלל וריאנטים (מידות/צדדים) - מסוכם לכל ערוץ. שורות בצבע אדום = התאמה לא-ודאית (כבר סומן בעבר). שורות/בלוקים בצבע כתום = אי-ודאות חדשה שעלתה בסריקה המורחבת - טרם הוכרעה, מוצגת לבירור מול המשתמש בנפרד, לא מסוכמת בטבלה הראשית.</t>
+    <t xml:space="preserve">תיקון (25/09/2026): בגרסה הקודמת נעשה שימוש בקוד CHEMIPAL המספרי (כמו 4411030) כמפתח חיפוש עבור דגמים שהותאמו דרך TRANS/הקטלוג (213 CTS, SH422, 397A, SH333) - זה תפס נכון מול 5 גיליונות CEMIUP0.9 (שם עמודת הקוד היא באמת הקוד המספרי), אבל פספס לגמרי את 29 גיליונות ה-SALES הישירים (שם עמודת "Product Code" מכילה את הקוד הטקסטואלי הגולמי כמו "213CTSR L", לא את הקוד המספרי) - בעיית אי-התאמת סוג-מפתח, לא בדיוק בעיית רווחים כפי שהועלתה. התיקון: סריקה חדשה לגמרי שמחפשת את קידומת-הבסיס הטקסטואלית (עם נרמול רווחים/מקפים/פלוס) ישירות מול עמודת הקוד הגולמית + שם המוצר בכל 34 המקורות (5 CEMIUP0.9 + 29 SALES, ללא 107/113 שכבר כלולות בתוך בתי מרקחת/מאוחדת - מניעת כפל ספירה). כמות/כסף = 2026 בפועל עד היום (YTD), לא מנורמל. כאשר דגם כלל וריאנטים (מידות/צדדים) - מסוכם לכל ערוץ. שורות בצבע אדום = התאמה לא-ודאית (T40B "רצועה לפיקה" - קוד דומה בלבד, סומן ולא הוכרע). עדכון 26/09/2026: כל 5 אי-הוודאויות שעלו בסריקה המורחבת (59 / 3051 x3 / MSG001F 0 / cervical collar) הוכרעו במפורש ע"י המשתמש ועודכנו בטבלה הראשית: "59", "3051" (×3) ו-"cervical collar" נקבעו כ-0 יחידות/NA (לא אותו מוצר, לא מוזג); "MSG001F 0" מוזג כעת מכל 3 גווני הצבע (שחור/קרם/לבן) יחד לשורה אחת מאוחדת, כולל שורת הזיכוי השלילית בגוון הלבן כפי שהיא בנתונים.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -227,10 +227,7 @@
     <t xml:space="preserve">-- סה"כ 809PW --</t>
   </si>
   <si>
-    <t xml:space="preserve">- (אי-ודאות, ראה גיליון תחתון)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">אי-ודאות שעלתה בסריקה המורחבת - ראה טבלת "אי-ודאויות לבירור" בתחתית</t>
+    <t xml:space="preserve">הוכרע ע"י המשתמש (26/09/2026): 0 יחידות ב-2026 - אף אחת מ-41 זהויות-הווריאנט שנמצאו עבור "59" אינה המוצר המבוקש, לא מוזג.</t>
   </si>
   <si>
     <t xml:space="preserve">T40B</t>
@@ -254,9 +251,21 @@
     <t xml:space="preserve">-- סה"כ T066 --</t>
   </si>
   <si>
+    <t xml:space="preserve">הוכרע ע"י המשתמש (26/09/2026): 0 יחידות ב-2026 - קוד CHEMIPAL 4413051 ("35 XXL מגן קרסול לבן") אינו אותו מוצר כמו "3051", לא מוזג.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הוכרע ע"י המשתמש (26/09/2026): זהה לשורה 16 (כפילות ברשימת המקור) - 0 יחידות, לא מוזג.</t>
+  </si>
+  <si>
     <t xml:space="preserve">MSG001F 0</t>
   </si>
   <si>
+    <t xml:space="preserve">הוכרע ע"י המשתמש (26/09/2026): מוזג סה"כ כל 3 גווני MSG001F (שחור/קרם/לבן) יחד, ללא הבחנה בצבע, כולל שורת הזיכוי השלילית בגוון הלבן כפי שהיא.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-- סה"כ MSG001F 0 --</t>
+  </si>
+  <si>
     <t xml:space="preserve">MSG002S 0</t>
   </si>
   <si>
@@ -278,6 +287,9 @@
     <t xml:space="preserve">cervical collar</t>
   </si>
   <si>
+    <t xml:space="preserve">הוכרע ע"י המשתמש (26/09/2026): 0 יחידות ב-2026 - אף אחת מ-3 משפחות ה"צווארון" שנמצאו (621B / 61BL / 60B) אינה ה-"cervical collar" המבוקש, לא מוזג.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Miami brace</t>
   </si>
   <si>
@@ -291,24 +303,6 @@
   </si>
   <si>
     <t xml:space="preserve">-- סה"כ T36B --</t>
-  </si>
-  <si>
-    <t xml:space="preserve">אי-ודאויות לבירור מול המשתמש (לא סוכמו/מוזגו אוטומטית)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">עמום מדי לזיהוי מוצר ספציפי: הבסיס "59" תואם 41 זהויות-וריאנט שונות (חגורות שבר בכל הצדדים/מידות, חלקן עם שורת זיכוי/החזרה שלילית) על פני כמעט כל קטגוריה - סה"כ גולמי ~381 יח'/71,042 ש"ח, אך לא סביר שזה כולו "מוצר אחד". לא מסוכם. דורש בירור: איזה צד/מידה בדיוק?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">לא נמצאה התאמה אמיתית. נמצא רק צירוף מספרים מקרי: קוד CHEMIPAL 4413051 ("35 XXL מגן קרסול לבן") מסתיים ב-"3051" בטעות סטטיסטית (213 יח'/5,099.97 ש"ח, 4 ערוצי CEMIUP) - כנראה לא אותו מוצר. דורש בירור.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">זהה לשורה 16 (כפילות ברשימת המקור) - אותה התאמה מקרית בלבד, לא מסוכמת.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">לא נמצאה התאמה מדויקת ל-"MSG001F 0" עצמו, אך נמצאה משפחה קרובה עם סיומות צבע: MSG001FB 0 (שחור, 33 יח'/26,246.27 ש"ח), MSG001FC (קרם, 14 יח'/12,201.54 ש"ח), MSG001FW (לבן, -1 יח'/-524.93 ש"ח - שורת זיכוי). לא ברור אם "MSG001F 0" ברשימה המקורית מתכוון למשפחה כולה או שזה קוד גנרי שלא נמכר בפועל בלי סיומת צבע. דורש בירור.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">לא נמצאה התאמה למילים האנגליות "cervical collar" ישירות, אך נמצאו 3 משפחות מוצר שונות בעברית שמכילות "צווארון" (=collar): (א) "621B" - Cervicallo IceSilk צווארון משי רך, 4 מידות, ~46 יח'/2,978 ש"ח, ערוצים 101/103/213-SPAIN; (ב) "61BL" - Cervicallo Soft צווארון ספוגי כחול, 4 מידות, ~11 יח'/375 ש"ח, ערוצים 101/103; (ג) "60B" - צווארון ספוג/צוארון ספוגי, 6 מידות, ~145 יח' נטו/6,821 ש"ח (כולל שורת זיכוי שלילית ב-XS), ערוצים 103/114/210-FINLAND/216-CYPRUS. יתכן שאחת מהן (או יותר) היא ה"cervical collar" המבוקש - לא ברור איזו, ולכן לא מוזג אוטומטית. דורש בירור.</t>
   </si>
 </sst>
 </file>
@@ -321,7 +315,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -408,13 +402,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FF7F6000"/>
       <name val="Arial"/>
@@ -432,7 +419,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -454,13 +441,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8CBAD"/>
-        <bgColor rgb="FFFFE699"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE699"/>
-        <bgColor rgb="FFF8CBAD"/>
+        <bgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -498,7 +479,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -631,6 +612,22 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -643,47 +640,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -733,7 +702,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFE699"/>
+      <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -2422,7 +2391,7 @@
         <v>59</v>
       </c>
       <c r="C76" s="12" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D76" s="23" t="s">
         <v>42</v>
@@ -2432,7 +2401,7 @@
       </c>
       <c r="F76" s="12"/>
       <c r="G76" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2440,7 +2409,7 @@
         <v>13</v>
       </c>
       <c r="B77" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C77" s="12" t="s">
         <v>11</v>
@@ -2461,7 +2430,7 @@
         <v>13</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C78" s="12" t="s">
         <v>38</v>
@@ -2482,7 +2451,7 @@
         <v>13</v>
       </c>
       <c r="B79" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C79" s="12" t="s">
         <v>19</v>
@@ -2503,7 +2472,7 @@
         <v>13</v>
       </c>
       <c r="B80" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C80" s="12" t="s">
         <v>17</v>
@@ -2524,7 +2493,7 @@
         <v>13</v>
       </c>
       <c r="B81" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C81" s="12" t="s">
         <v>21</v>
@@ -2545,7 +2514,7 @@
         <v>13</v>
       </c>
       <c r="B82" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C82" s="12" t="s">
         <v>22</v>
@@ -2566,10 +2535,10 @@
         <v>13</v>
       </c>
       <c r="B83" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C83" s="29" t="s">
         <v>53</v>
-      </c>
-      <c r="C83" s="29" t="s">
-        <v>54</v>
       </c>
       <c r="D83" s="30" t="n">
         <v>8</v>
@@ -2579,13 +2548,13 @@
       </c>
       <c r="F83" s="28"/>
       <c r="G83" s="32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="19"/>
       <c r="B84" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C84" s="19"/>
       <c r="D84" s="16" t="n">
@@ -2597,255 +2566,255 @@
       <c r="F84" s="19"/>
       <c r="G84" s="19"/>
     </row>
-    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="33" t="n">
+    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="B85" s="33" t="s">
+      <c r="B85" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C85" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D85" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="E85" s="9" t="n">
+        <v>3198.69</v>
+      </c>
+      <c r="F85" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" s="10"/>
+    </row>
+    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B86" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C86" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D86" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="E86" s="9" t="n">
+        <v>333.98</v>
+      </c>
+      <c r="F86" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="10"/>
+    </row>
+    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B87" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C87" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D87" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E87" s="9" t="n">
+        <v>588.13</v>
+      </c>
+      <c r="F87" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="10"/>
+    </row>
+    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A88" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B88" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C88" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D88" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" s="9" t="n">
+        <v>85.26</v>
+      </c>
+      <c r="F88" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A89" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B89" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C89" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D89" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F89" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G89" s="10"/>
+    </row>
+    <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B90" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C90" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D90" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E90" s="9" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F90" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G90" s="10"/>
+    </row>
+    <row r="91" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A91" s="28" t="n">
+        <v>14</v>
+      </c>
+      <c r="B91" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C91" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="C85" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="D85" s="34" t="n">
-        <v>22</v>
-      </c>
-      <c r="E85" s="35" t="n">
-        <v>3198.69</v>
-      </c>
-      <c r="F85" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G85" s="10"/>
-    </row>
-    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="33" t="n">
-        <v>14</v>
-      </c>
-      <c r="B86" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="C86" s="33" t="s">
+      <c r="D91" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="E91" s="31" t="n">
+        <v>588.13</v>
+      </c>
+      <c r="F91" s="28"/>
+      <c r="G91" s="32" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="19"/>
+      <c r="B92" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C92" s="19"/>
+      <c r="D92" s="16" t="n">
+        <v>51</v>
+      </c>
+      <c r="E92" s="14" t="n">
+        <v>4794.24</v>
+      </c>
+      <c r="F92" s="19"/>
+      <c r="G92" s="19"/>
+    </row>
+    <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A93" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B93" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C93" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D93" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E93" s="9" t="n">
+        <v>568.56</v>
+      </c>
+      <c r="F93" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G93" s="10"/>
+    </row>
+    <row r="94" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A94" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B94" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C94" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D94" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F94" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G94" s="10"/>
+    </row>
+    <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B95" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C95" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D86" s="34" t="n">
-        <v>10</v>
-      </c>
-      <c r="E86" s="35" t="n">
-        <v>333.98</v>
-      </c>
-      <c r="F86" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G86" s="10"/>
-    </row>
-    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="33" t="n">
-        <v>14</v>
-      </c>
-      <c r="B87" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="C87" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="D87" s="34" t="n">
-        <v>8</v>
-      </c>
-      <c r="E87" s="35" t="n">
-        <v>588.13</v>
-      </c>
-      <c r="F87" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G87" s="10"/>
-    </row>
-    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="33" t="n">
-        <v>14</v>
-      </c>
-      <c r="B88" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="C88" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="D88" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E88" s="35" t="n">
-        <v>85.26</v>
-      </c>
-      <c r="F88" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G88" s="10"/>
-    </row>
-    <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="33" t="n">
-        <v>14</v>
-      </c>
-      <c r="B89" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="C89" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="D89" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E89" s="35" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F89" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G89" s="10"/>
-    </row>
-    <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="33" t="n">
-        <v>14</v>
-      </c>
-      <c r="B90" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="C90" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="D90" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E90" s="35" t="n">
+      <c r="D95" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" s="9" t="n">
         <v>0.03</v>
       </c>
-      <c r="F90" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G90" s="10"/>
-    </row>
-    <row r="91" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="36" t="n">
-        <v>14</v>
-      </c>
-      <c r="B91" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="C91" s="37" t="s">
-        <v>54</v>
-      </c>
-      <c r="D91" s="38" t="n">
-        <v>8</v>
-      </c>
-      <c r="E91" s="39" t="n">
-        <v>588.13</v>
-      </c>
-      <c r="F91" s="36"/>
-      <c r="G91" s="32" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="40"/>
-      <c r="B92" s="41" t="s">
-        <v>57</v>
-      </c>
-      <c r="C92" s="40"/>
-      <c r="D92" s="42" t="n">
-        <v>51</v>
-      </c>
-      <c r="E92" s="43" t="n">
-        <v>4794.24</v>
-      </c>
-      <c r="F92" s="40"/>
-      <c r="G92" s="40"/>
-    </row>
-    <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="33" t="n">
-        <v>15</v>
-      </c>
-      <c r="B93" s="33" t="s">
+      <c r="F95" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" s="10"/>
+    </row>
+    <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A96" s="19"/>
+      <c r="B96" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="C93" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="D93" s="34" t="n">
-        <v>4</v>
-      </c>
-      <c r="E93" s="35" t="n">
-        <v>568.56</v>
-      </c>
-      <c r="F93" s="33" t="n">
-        <v>2</v>
-      </c>
-      <c r="G93" s="10"/>
-    </row>
-    <row r="94" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="33" t="n">
-        <v>15</v>
-      </c>
-      <c r="B94" s="33" t="s">
-        <v>58</v>
-      </c>
-      <c r="C94" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="D94" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E94" s="35" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F94" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G94" s="10"/>
-    </row>
-    <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="33" t="n">
-        <v>15</v>
-      </c>
-      <c r="B95" s="33" t="s">
-        <v>58</v>
-      </c>
-      <c r="C95" s="33" t="s">
-        <v>38</v>
-      </c>
-      <c r="D95" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E95" s="35" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="F95" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G95" s="10"/>
-    </row>
-    <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="40"/>
-      <c r="B96" s="41" t="s">
-        <v>59</v>
-      </c>
-      <c r="C96" s="40"/>
-      <c r="D96" s="42" t="n">
+      <c r="C96" s="19"/>
+      <c r="D96" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="E96" s="43" t="n">
+      <c r="E96" s="14" t="n">
         <v>568.6</v>
       </c>
-      <c r="F96" s="40"/>
-      <c r="G96" s="40"/>
-    </row>
-    <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="33" t="n">
+      <c r="F96" s="19"/>
+      <c r="G96" s="19"/>
+    </row>
+    <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A97" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B97" s="33" t="n">
+      <c r="B97" s="12" t="n">
         <v>3051</v>
       </c>
-      <c r="C97" s="33" t="s">
-        <v>51</v>
+      <c r="C97" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="D97" s="23" t="s">
         <v>42</v>
@@ -2853,20 +2822,20 @@
       <c r="E97" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="F97" s="33"/>
+      <c r="F97" s="12"/>
       <c r="G97" s="10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="33" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A98" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B98" s="33" t="n">
+      <c r="B98" s="12" t="n">
         <v>3051</v>
       </c>
-      <c r="C98" s="33" t="s">
-        <v>51</v>
+      <c r="C98" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="D98" s="23" t="s">
         <v>42</v>
@@ -2874,20 +2843,20 @@
       <c r="E98" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="F98" s="33"/>
+      <c r="F98" s="12"/>
       <c r="G98" s="10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="33" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B99" s="33" t="n">
+      <c r="B99" s="12" t="n">
         <v>3051</v>
       </c>
-      <c r="C99" s="33" t="s">
-        <v>51</v>
+      <c r="C99" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="D99" s="23" t="s">
         <v>42</v>
@@ -2895,224 +2864,220 @@
       <c r="E99" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="F99" s="33"/>
+      <c r="F99" s="12"/>
       <c r="G99" s="10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="33" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B100" s="33" t="s">
-        <v>60</v>
-      </c>
-      <c r="C100" s="33" t="s">
-        <v>51</v>
-      </c>
-      <c r="D100" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="E100" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="F100" s="33"/>
+      <c r="B100" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C100" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D100" s="20" t="n">
+        <v>37</v>
+      </c>
+      <c r="E100" s="21" t="n">
+        <v>34302.36</v>
+      </c>
+      <c r="F100" s="12" t="n">
+        <v>2</v>
+      </c>
       <c r="G100" s="10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="33" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A101" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="B101" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C101" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D101" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E101" s="9" t="n">
+        <v>2624.65</v>
+      </c>
+      <c r="F101" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G101" s="10"/>
+    </row>
+    <row r="102" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="B102" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C102" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D102" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E102" s="9" t="n">
+        <v>508.43</v>
+      </c>
+      <c r="F102" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G102" s="10"/>
+    </row>
+    <row r="103" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A103" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="B103" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C103" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B101" s="33" t="s">
-        <v>61</v>
-      </c>
-      <c r="C101" s="33" t="s">
+      <c r="D103" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" s="9" t="n">
+        <v>487.44</v>
+      </c>
+      <c r="F103" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" s="10"/>
+    </row>
+    <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A104" s="17"/>
+      <c r="B104" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C104" s="17"/>
+      <c r="D104" s="16" t="n">
+        <v>46</v>
+      </c>
+      <c r="E104" s="14" t="n">
+        <v>37922.88</v>
+      </c>
+      <c r="F104" s="17"/>
+      <c r="G104" s="15"/>
+    </row>
+    <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A105" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="B105" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C105" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D101" s="34" t="n">
+      <c r="D105" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="E101" s="35" t="n">
+      <c r="E105" s="9" t="n">
         <v>16626.44</v>
       </c>
-      <c r="F101" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G101" s="10"/>
-    </row>
-    <row r="102" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="33" t="n">
+      <c r="F105" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" s="10"/>
+    </row>
+    <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A106" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B102" s="33" t="s">
-        <v>61</v>
-      </c>
-      <c r="C102" s="33" t="s">
+      <c r="B106" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C106" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D102" s="34" t="n">
+      <c r="D106" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="E102" s="35" t="n">
+      <c r="E106" s="21" t="n">
         <v>4199.44</v>
       </c>
-      <c r="F102" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G102" s="10"/>
-    </row>
-    <row r="103" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="33" t="n">
+      <c r="F106" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G106" s="10"/>
+    </row>
+    <row r="107" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A107" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B103" s="33" t="s">
-        <v>61</v>
-      </c>
-      <c r="C103" s="33" t="s">
+      <c r="B107" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C107" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D103" s="34" t="n">
+      <c r="D107" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="E103" s="35" t="n">
+      <c r="E107" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="F103" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G103" s="10"/>
-    </row>
-    <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="33" t="n">
+      <c r="F107" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G107" s="10"/>
+    </row>
+    <row r="108" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A108" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B104" s="33" t="s">
-        <v>61</v>
-      </c>
-      <c r="C104" s="33" t="s">
+      <c r="B108" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C108" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D104" s="34" t="n">
+      <c r="D108" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="E104" s="35" t="n">
+      <c r="E108" s="21" t="n">
         <v>1012.36</v>
       </c>
-      <c r="F104" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G104" s="10"/>
-    </row>
-    <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="40"/>
-      <c r="B105" s="41" t="s">
-        <v>62</v>
-      </c>
-      <c r="C105" s="40"/>
-      <c r="D105" s="42" t="n">
+      <c r="F108" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G108" s="10"/>
+    </row>
+    <row r="109" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="17"/>
+      <c r="B109" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C109" s="17"/>
+      <c r="D109" s="24" t="n">
         <v>30</v>
       </c>
-      <c r="E105" s="43" t="n">
+      <c r="E109" s="25" t="n">
         <v>21838.24</v>
       </c>
-      <c r="F105" s="40"/>
-      <c r="G105" s="40"/>
-    </row>
-    <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="33" t="n">
+      <c r="F109" s="17"/>
+      <c r="G109" s="15"/>
+    </row>
+    <row r="110" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A110" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="B106" s="33" t="s">
-        <v>63</v>
-      </c>
-      <c r="C106" s="33" t="s">
+      <c r="B110" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C110" s="12" t="s">
         <v>41</v>
-      </c>
-      <c r="D106" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="E106" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="F106" s="33"/>
-      <c r="G106" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="107" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="33" t="n">
-        <v>22</v>
-      </c>
-      <c r="B107" s="33" t="s">
-        <v>64</v>
-      </c>
-      <c r="C107" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="D107" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="E107" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="F107" s="33"/>
-      <c r="G107" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="108" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="33" t="n">
-        <v>23</v>
-      </c>
-      <c r="B108" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="C108" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="D108" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="E108" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="F108" s="33"/>
-      <c r="G108" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="109" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="33" t="n">
-        <v>24</v>
-      </c>
-      <c r="B109" s="33" t="s">
-        <v>66</v>
-      </c>
-      <c r="C109" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="D109" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="E109" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="F109" s="33"/>
-      <c r="G109" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="33" t="n">
-        <v>25</v>
-      </c>
-      <c r="B110" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C110" s="33" t="s">
-        <v>51</v>
       </c>
       <c r="D110" s="23" t="s">
         <v>42</v>
@@ -3120,19 +3085,19 @@
       <c r="E110" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="F110" s="33"/>
+      <c r="F110" s="12"/>
       <c r="G110" s="10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="111" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="33" t="n">
-        <v>26</v>
-      </c>
-      <c r="B111" s="33" t="s">
-        <v>68</v>
-      </c>
-      <c r="C111" s="33" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A111" s="12" t="n">
+        <v>22</v>
+      </c>
+      <c r="B111" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C111" s="12" t="s">
         <v>41</v>
       </c>
       <c r="D111" s="23" t="s">
@@ -3141,250 +3106,253 @@
       <c r="E111" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="F111" s="33"/>
+      <c r="F111" s="12"/>
       <c r="G111" s="10" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="33" t="n">
+    <row r="112" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A112" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="B112" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C112" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D112" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="E112" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="F112" s="12"/>
+      <c r="G112" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A113" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="B113" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C113" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D113" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="E113" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="F113" s="12"/>
+      <c r="G113" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A114" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="B114" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="C114" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D114" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="E114" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="F114" s="12"/>
+      <c r="G114" s="10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A115" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="B115" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C115" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D115" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="E115" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="F115" s="12"/>
+      <c r="G115" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A116" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="B112" s="33" t="s">
-        <v>69</v>
-      </c>
-      <c r="C112" s="33" t="s">
+      <c r="B116" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C116" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D112" s="34" t="n">
+      <c r="D116" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="E112" s="35" t="n">
+      <c r="E116" s="9" t="n">
         <v>406.01</v>
       </c>
-      <c r="F112" s="33" t="n">
+      <c r="F116" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="G112" s="10"/>
-    </row>
-    <row r="113" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="33" t="n">
+      <c r="G116" s="10"/>
+    </row>
+    <row r="117" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A117" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="B113" s="33" t="s">
-        <v>69</v>
-      </c>
-      <c r="C113" s="33" t="s">
+      <c r="B117" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C117" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D113" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E113" s="35" t="n">
+      <c r="D117" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E117" s="9" t="n">
         <v>0.01</v>
       </c>
-      <c r="F113" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G113" s="10"/>
-    </row>
-    <row r="114" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="33" t="n">
+      <c r="F117" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G117" s="10"/>
+    </row>
+    <row r="118" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A118" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="B114" s="33" t="s">
-        <v>69</v>
-      </c>
-      <c r="C114" s="33" t="s">
+      <c r="B118" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C118" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D114" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E114" s="35" t="n">
+      <c r="D118" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E118" s="9" t="n">
         <v>0.03</v>
       </c>
-      <c r="F114" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G114" s="10"/>
-    </row>
-    <row r="115" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="40"/>
-      <c r="B115" s="41" t="s">
-        <v>70</v>
-      </c>
-      <c r="C115" s="40"/>
-      <c r="D115" s="42" t="n">
+      <c r="F118" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G118" s="10"/>
+    </row>
+    <row r="119" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="33"/>
+      <c r="B119" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="C119" s="33"/>
+      <c r="D119" s="35" t="n">
         <v>7</v>
       </c>
-      <c r="E115" s="43" t="n">
+      <c r="E119" s="36" t="n">
         <v>406.05</v>
       </c>
-      <c r="F115" s="40"/>
-      <c r="G115" s="40"/>
-    </row>
-    <row r="116" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="33" t="n">
+      <c r="F119" s="33"/>
+      <c r="G119" s="33"/>
+    </row>
+    <row r="120" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A120" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="B116" s="33" t="s">
-        <v>71</v>
-      </c>
-      <c r="C116" s="33" t="s">
+      <c r="B120" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="C120" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="D116" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E116" s="35" t="n">
+      <c r="D120" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E120" s="39" t="n">
         <v>0.01</v>
       </c>
-      <c r="F116" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G116" s="10"/>
-    </row>
-    <row r="117" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="33" t="n">
+      <c r="F120" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G120" s="10"/>
+    </row>
+    <row r="121" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A121" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="B117" s="33" t="s">
-        <v>71</v>
-      </c>
-      <c r="C117" s="33" t="s">
+      <c r="B121" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C121" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="D117" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E117" s="35" t="n">
+      <c r="D121" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E121" s="39" t="n">
         <v>0.03</v>
       </c>
-      <c r="F117" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G117" s="10"/>
-    </row>
-    <row r="118" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="40"/>
-      <c r="B118" s="41" t="s">
-        <v>72</v>
-      </c>
-      <c r="C118" s="40"/>
-      <c r="D118" s="42" t="n">
+      <c r="F121" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G121" s="10"/>
+    </row>
+    <row r="122" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A122" s="40"/>
+      <c r="B122" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="C122" s="41"/>
+      <c r="D122" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="E118" s="43" t="n">
+      <c r="E122" s="36" t="n">
         <v>0.04</v>
       </c>
-      <c r="F118" s="40"/>
-      <c r="G118" s="40"/>
-    </row>
-    <row r="120" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="44" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="121" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A121" s="45" t="n">
-        <v>12</v>
-      </c>
-      <c r="B121" s="45" t="n">
-        <v>59</v>
-      </c>
-      <c r="C121" s="46" t="s">
-        <v>74</v>
-      </c>
-      <c r="D121" s="46"/>
-      <c r="E121" s="46"/>
-      <c r="F121" s="46"/>
-      <c r="G121" s="46"/>
-    </row>
-    <row r="122" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A122" s="45" t="n">
-        <v>16</v>
-      </c>
-      <c r="B122" s="45" t="n">
-        <v>3051</v>
-      </c>
-      <c r="C122" s="46" t="s">
-        <v>75</v>
-      </c>
-      <c r="D122" s="46"/>
-      <c r="E122" s="46"/>
-      <c r="F122" s="46"/>
-      <c r="G122" s="46"/>
+      <c r="F122" s="33"/>
+      <c r="G122" s="33"/>
     </row>
     <row r="123" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A123" s="45" t="n">
-        <v>17</v>
-      </c>
-      <c r="B123" s="45" t="n">
-        <v>3051</v>
-      </c>
-      <c r="C123" s="46" t="s">
-        <v>76</v>
-      </c>
-      <c r="D123" s="46"/>
-      <c r="E123" s="46"/>
-      <c r="F123" s="46"/>
-      <c r="G123" s="46"/>
+      <c r="A123" s="42"/>
+      <c r="B123" s="42"/>
+      <c r="C123" s="43"/>
     </row>
     <row r="124" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A124" s="45" t="n">
-        <v>18</v>
-      </c>
-      <c r="B124" s="45" t="n">
-        <v>3051</v>
-      </c>
-      <c r="C124" s="46" t="s">
-        <v>76</v>
-      </c>
-      <c r="D124" s="46"/>
-      <c r="E124" s="46"/>
-      <c r="F124" s="46"/>
-      <c r="G124" s="46"/>
+      <c r="A124" s="42"/>
+      <c r="B124" s="42"/>
+      <c r="C124" s="43"/>
     </row>
     <row r="125" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A125" s="45" t="n">
-        <v>19</v>
-      </c>
-      <c r="B125" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="C125" s="46" t="s">
-        <v>77</v>
-      </c>
-      <c r="D125" s="46"/>
-      <c r="E125" s="46"/>
-      <c r="F125" s="46"/>
-      <c r="G125" s="46"/>
+      <c r="A125" s="42"/>
+      <c r="B125" s="42"/>
+      <c r="C125" s="43"/>
     </row>
     <row r="126" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A126" s="45" t="n">
-        <v>25</v>
-      </c>
-      <c r="B126" s="45" t="s">
-        <v>67</v>
-      </c>
-      <c r="C126" s="46" t="s">
-        <v>78</v>
-      </c>
-      <c r="D126" s="46"/>
-      <c r="E126" s="46"/>
-      <c r="F126" s="46"/>
-      <c r="G126" s="46"/>
+      <c r="A126" s="42"/>
+      <c r="B126" s="42"/>
+      <c r="C126" s="43"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="1">
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="C121:G121"/>
-    <mergeCell ref="C122:G122"/>
-    <mergeCell ref="C123:G123"/>
-    <mergeCell ref="C124:G124"/>
-    <mergeCell ref="C125:G125"/>
-    <mergeCell ref="C126:G126"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add Plan vs Actual sheet to new-products-match
New "Plan vs Actual" sheet compares the corrected 2026 target file
(quantity/price/sales/channel per model) against YTD actual from the
existing long-format table, with an explicit note that actual is
partial-year (~9.5 months) vs a full 12-month plan target. 28
rows, matching the original list's duplicates (T40B x2, 3051 x3)
individually. Totals: 16,380 planned vs 8,220 actual units (50.2%),
₪1,434,906 planned vs ₪667,610.16 actual (46.5%). 9 models at 0%
execution. Channel comparison: only SH776 matches its planned
channel exactly; 14 models sold through a different channel than
planned (e.g. 213 CTS planned for Orthopedic institutes, actually
led by IL online). Long-format "גיליון1" table unchanged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QvuhBZminJvrtKVH8YY8
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-09-25-new-products-match.xlsx
+++ b/kirill/outputs/2026-09-25-new-products-match.xlsx
@@ -9,6 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Plan vs Actual" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -72,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="110">
   <si>
     <t xml:space="preserve">מוצרים חדשים - התאמת כמות/כסף 2026 בפועל (YTD) לפי ערוץ מכירה - גרסה סופית (כל 5 אי-הוודאויות הוכרעו ע"י המשתמש)</t>
   </si>
@@ -303,19 +304,119 @@
   </si>
   <si>
     <t xml:space="preserve">-- סה"כ T36B --</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan vs Actual - תוכנית 2026 מול ביצוע בפועל (YTD) למוצרים חדשים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אזהרה מתודולוגית חשובה: עמודות התוכנית (C-F) הן יעד ל-2026 המלאה (12 חודשים). עמודות הבפועל (G-I) הן YTD חלקי בלבד (כפי שמחושב בגיליון "גיליון1" - מבוסס על ~9.5 חודשי נתונים בפועל, לא מנורמל לשנה מלאה כאן בכוונה, כדי להשוות "מה כבר נמכר בפועל" מול "היעד השנתי" ישירות). % הביצוע (K-L) הוא לכן ביחס ליעד שנתי מלא בעוד שהמונה הוא רק חלק מהשנה - לכן % נמוך (למשל 30-60%) בשלב הזה של השנה אינו בהכרח "פיגור", אלא צפוי אם קצב המכירות המנורמל עדיין תואם/עולה על היעד. T40B ו-3051 מופיעים כל אחד 2-3 פעמים ברשימת המקור (מופעים נפרדים עם ערוצי-יעד שונים) - ה-actual זהה בשני מופעי T40B (הנתון הגולמי לא ניתן לפיצול בין המופעים) ולכן בשורת הסה"כ הכללי בתחתית, ה-actual של T40B נספר פעם אחת בלבד (לא כפול) כדי לא לנפח את הביצוע בפועל - הפלאן עדיין מסוכם משני המופעים כפי שהם. 3051 = 0 בפועל בכל 3 המופעים (הוכרע ע"י המשתמש כמוצר לא-זהה) - לא רלוונטי לכפל.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">דגם</t>
+  </si>
+  <si>
+    <t xml:space="preserve">כמות מתוכננת (שנתי)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מחיר ליח' (₪)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מכירות מתוכננות (שנתי, ₪)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ערוץ מתוכנן</t>
+  </si>
+  <si>
+    <t xml:space="preserve">כמות בפועל (YTD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">כסף בפועל (YTD, ₪)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ערוץ מוביל בפועל (Top Source)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ערוץ תואם?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% ביצוע כמות (YTD/יעד שנתי)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% ביצוע כסף (YTD/יעד שנתי)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מכוני אורטופדיה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">שונה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">סופרפארם</t>
+  </si>
+  <si>
+    <t xml:space="preserve">כמעט תיקו מול סופר פארם ישראל (1552, הפרש 18 יח' בלבד)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">תואם</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NA (0 בפועל)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אין בפועל (0%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אין ערוץ מתוכנן</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T40B (מופע 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">כולל 8 יח'/588.13 ש"ח משורה לא-ודאית ("T40B רצועה לפיקה")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T40B (מופע 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3051 (מופע 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3051 (מופע 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3051 (מופע 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">101-Factory customers / 207-Salus HUNGARY (תיקו)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">תיקו בין 2 ערוצים - 1 יח' כל אחד, אין ערוץ מוביל יחיד</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-- סה"כ (כל 28 שורות התוכנית, plan ללא כפל) --</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-- סה"כ מתוקן (T40B נספר פעם אחת - לא כפול) --</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -418,8 +519,16 @@
       <name val="FreeSans"/>
       <family val="2"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -435,12 +544,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE7E6E6"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFEDEDED"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8CBAD"/>
+        <bgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6E0B4"/>
+        <bgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDEDED"/>
         <bgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
@@ -479,7 +600,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="54">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -612,6 +733,70 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -628,32 +813,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -681,12 +842,12 @@
       <rgbColor rgb="FF7F6000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFC6E0B4"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFEDEDED"/>
       <rgbColor rgb="FFE7E6E6"/>
-      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -3258,38 +3419,38 @@
       </c>
       <c r="G118" s="10"/>
     </row>
-    <row r="119" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="33"/>
-      <c r="B119" s="34" t="s">
+    <row r="119" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A119" s="19"/>
+      <c r="B119" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="C119" s="33"/>
-      <c r="D119" s="35" t="n">
+      <c r="C119" s="19"/>
+      <c r="D119" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="E119" s="36" t="n">
+      <c r="E119" s="14" t="n">
         <v>406.05</v>
       </c>
-      <c r="F119" s="33"/>
-      <c r="G119" s="33"/>
+      <c r="F119" s="19"/>
+      <c r="G119" s="19"/>
     </row>
     <row r="120" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="B120" s="37" t="s">
+      <c r="B120" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="C120" s="37" t="s">
+      <c r="C120" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D120" s="38" t="n">
-        <v>1</v>
-      </c>
-      <c r="E120" s="39" t="n">
+      <c r="D120" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E120" s="9" t="n">
         <v>0.01</v>
       </c>
-      <c r="F120" s="37" t="n">
+      <c r="F120" s="12" t="n">
         <v>1</v>
       </c>
       <c r="G120" s="10"/>
@@ -3304,51 +3465,51 @@
       <c r="C121" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="D121" s="38" t="n">
-        <v>1</v>
-      </c>
-      <c r="E121" s="39" t="n">
+      <c r="D121" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E121" s="9" t="n">
         <v>0.03</v>
       </c>
-      <c r="F121" s="37" t="n">
+      <c r="F121" s="12" t="n">
         <v>1</v>
       </c>
       <c r="G121" s="10"/>
     </row>
     <row r="122" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A122" s="40"/>
+      <c r="A122" s="33"/>
       <c r="B122" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="C122" s="41"/>
-      <c r="D122" s="35" t="n">
+      <c r="C122" s="34"/>
+      <c r="D122" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E122" s="36" t="n">
+      <c r="E122" s="14" t="n">
         <v>0.04</v>
       </c>
-      <c r="F122" s="33"/>
-      <c r="G122" s="33"/>
+      <c r="F122" s="19"/>
+      <c r="G122" s="19"/>
     </row>
     <row r="123" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A123" s="42"/>
-      <c r="B123" s="42"/>
-      <c r="C123" s="43"/>
+      <c r="A123" s="35"/>
+      <c r="B123" s="35"/>
+      <c r="C123" s="36"/>
     </row>
     <row r="124" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A124" s="42"/>
-      <c r="B124" s="42"/>
-      <c r="C124" s="43"/>
+      <c r="A124" s="35"/>
+      <c r="B124" s="35"/>
+      <c r="C124" s="36"/>
     </row>
     <row r="125" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A125" s="42"/>
-      <c r="B125" s="42"/>
-      <c r="C125" s="43"/>
+      <c r="A125" s="35"/>
+      <c r="B125" s="35"/>
+      <c r="C125" s="36"/>
     </row>
     <row r="126" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A126" s="42"/>
-      <c r="B126" s="42"/>
-      <c r="C126" s="43"/>
+      <c r="A126" s="35"/>
+      <c r="B126" s="35"/>
+      <c r="C126" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3363,4 +3524,1264 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M36"/>
+  <sheetFormatPr defaultColWidth="8.6171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="37" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="39" t="n">
+        <v>46290</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="43.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="40" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="40" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" s="40" t="s">
+        <v>82</v>
+      </c>
+      <c r="F5" s="40" t="s">
+        <v>83</v>
+      </c>
+      <c r="G5" s="40" t="s">
+        <v>84</v>
+      </c>
+      <c r="H5" s="40" t="s">
+        <v>85</v>
+      </c>
+      <c r="I5" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="J5" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="L5" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="M5" s="40" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="42" t="n">
+        <v>2160</v>
+      </c>
+      <c r="D6" s="43" t="n">
+        <v>90</v>
+      </c>
+      <c r="E6" s="43" t="n">
+        <v>194400</v>
+      </c>
+      <c r="F6" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G6" s="42" t="n">
+        <v>1135</v>
+      </c>
+      <c r="H6" s="43" t="n">
+        <v>112752.57</v>
+      </c>
+      <c r="I6" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="J6" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K6" s="45" t="n">
+        <v>0.525462962962963</v>
+      </c>
+      <c r="L6" s="45" t="n">
+        <v>0.580002932098766</v>
+      </c>
+      <c r="M6" s="10"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="42" t="n">
+        <v>2880</v>
+      </c>
+      <c r="D7" s="43" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" s="43" t="n">
+        <v>288000</v>
+      </c>
+      <c r="F7" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="42" t="n">
+        <v>862</v>
+      </c>
+      <c r="H7" s="43" t="n">
+        <v>127955.57</v>
+      </c>
+      <c r="I7" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K7" s="45" t="n">
+        <v>0.299305555555556</v>
+      </c>
+      <c r="L7" s="45" t="n">
+        <v>0.444290173611111</v>
+      </c>
+      <c r="M7" s="10"/>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="42" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D8" s="43" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" s="43" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F8" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="G8" s="42" t="n">
+        <v>5823</v>
+      </c>
+      <c r="H8" s="43" t="n">
+        <v>306760.51</v>
+      </c>
+      <c r="I8" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K8" s="45" t="n">
+        <v>2.9115</v>
+      </c>
+      <c r="L8" s="45" t="n">
+        <v>3.0676051</v>
+      </c>
+      <c r="M8" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="41" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="42" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D9" s="43" t="n">
+        <v>70</v>
+      </c>
+      <c r="E9" s="43" t="n">
+        <v>70000</v>
+      </c>
+      <c r="F9" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G9" s="42" t="n">
+        <v>131</v>
+      </c>
+      <c r="H9" s="43" t="n">
+        <v>13889.9</v>
+      </c>
+      <c r="I9" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K9" s="45" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="L9" s="45" t="n">
+        <v>0.198427142857143</v>
+      </c>
+      <c r="M9" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="41" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="41" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="42" t="n">
+        <v>220</v>
+      </c>
+      <c r="D10" s="43" t="n">
+        <v>350</v>
+      </c>
+      <c r="E10" s="43" t="n">
+        <v>77000</v>
+      </c>
+      <c r="F10" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G10" s="42" t="n">
+        <v>103</v>
+      </c>
+      <c r="H10" s="43" t="n">
+        <v>40501.05</v>
+      </c>
+      <c r="I10" s="41" t="s">
+        <v>17</v>
+      </c>
+      <c r="J10" s="46" t="s">
+        <v>95</v>
+      </c>
+      <c r="K10" s="45" t="n">
+        <v>0.468181818181818</v>
+      </c>
+      <c r="L10" s="45" t="n">
+        <v>0.525987662337662</v>
+      </c>
+      <c r="M10" s="10"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="42" t="n">
+        <v>280</v>
+      </c>
+      <c r="D11" s="43" t="n">
+        <v>70</v>
+      </c>
+      <c r="E11" s="43" t="n">
+        <v>19600</v>
+      </c>
+      <c r="F11" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G11" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="43" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I11" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="J11" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K11" s="45" t="n">
+        <v>0.00357142857142857</v>
+      </c>
+      <c r="L11" s="45" t="n">
+        <v>1.53061224489796E-006</v>
+      </c>
+      <c r="M11" s="10"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="41" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="41" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="42" t="n">
+        <v>280</v>
+      </c>
+      <c r="D12" s="43" t="n">
+        <v>80</v>
+      </c>
+      <c r="E12" s="43" t="n">
+        <v>22400</v>
+      </c>
+      <c r="F12" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G12" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J12" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="K12" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="10"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="41" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="D13" s="43" t="n">
+        <v>260</v>
+      </c>
+      <c r="E13" s="43" t="n">
+        <v>52000</v>
+      </c>
+      <c r="F13" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G13" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="43" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I13" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="J13" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K13" s="45" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L13" s="45" t="n">
+        <v>5.76923076923077E-007</v>
+      </c>
+      <c r="M13" s="10"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="41" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="42" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D14" s="43" t="n">
+        <v>24</v>
+      </c>
+      <c r="E14" s="43" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F14" s="41" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="H14" s="43" t="n">
+        <v>50.25</v>
+      </c>
+      <c r="I14" s="41" t="s">
+        <v>20</v>
+      </c>
+      <c r="J14" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K14" s="45" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="L14" s="45" t="n">
+        <v>0.00209375</v>
+      </c>
+      <c r="M14" s="10"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="41" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="41" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D15" s="43" t="n">
+        <v>130</v>
+      </c>
+      <c r="E15" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="G15" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J15" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="K15" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="L15" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="M15" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="41" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="41" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="42" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D16" s="43" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" s="43" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F16" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" s="42" t="n">
+        <v>16</v>
+      </c>
+      <c r="H16" s="43" t="n">
+        <v>170.2</v>
+      </c>
+      <c r="I16" s="41" t="s">
+        <v>20</v>
+      </c>
+      <c r="J16" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K16" s="45" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="L16" s="45" t="n">
+        <v>0.00709166666666667</v>
+      </c>
+      <c r="M16" s="10"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="41" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="41" t="n">
+        <v>59</v>
+      </c>
+      <c r="C17" s="42" t="n">
+        <v>500</v>
+      </c>
+      <c r="D17" s="43" t="n">
+        <v>150</v>
+      </c>
+      <c r="E17" s="43" t="n">
+        <v>75000</v>
+      </c>
+      <c r="F17" s="47" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J17" s="48" t="s">
+        <v>99</v>
+      </c>
+      <c r="K17" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="10"/>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="41" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="41" t="s">
+        <v>100</v>
+      </c>
+      <c r="C18" s="42" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D18" s="43" t="n">
+        <v>60.61</v>
+      </c>
+      <c r="E18" s="43" t="n">
+        <v>60606</v>
+      </c>
+      <c r="F18" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="42" t="n">
+        <v>51</v>
+      </c>
+      <c r="H18" s="43" t="n">
+        <v>4794.24</v>
+      </c>
+      <c r="I18" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="J18" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K18" s="45" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="L18" s="45" t="n">
+        <v>0.0791050391050391</v>
+      </c>
+      <c r="M18" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="41" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="41" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="D19" s="43" t="n">
+        <v>70</v>
+      </c>
+      <c r="E19" s="43" t="n">
+        <v>21000</v>
+      </c>
+      <c r="F19" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G19" s="42" t="n">
+        <v>51</v>
+      </c>
+      <c r="H19" s="43" t="n">
+        <v>4794.24</v>
+      </c>
+      <c r="I19" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="J19" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K19" s="45" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="L19" s="45" t="n">
+        <v>0.228297142857143</v>
+      </c>
+      <c r="M19" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="41" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="41" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="D20" s="43" t="n">
+        <v>140</v>
+      </c>
+      <c r="E20" s="43" t="n">
+        <v>42000</v>
+      </c>
+      <c r="F20" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G20" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" s="43" t="n">
+        <v>568.6</v>
+      </c>
+      <c r="I20" s="41" t="s">
+        <v>20</v>
+      </c>
+      <c r="J20" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K20" s="45" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="L20" s="45" t="n">
+        <v>0.0135380952380952</v>
+      </c>
+      <c r="M20" s="10"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="41" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="C21" s="42" t="n">
+        <v>500</v>
+      </c>
+      <c r="D21" s="43" t="n">
+        <v>75</v>
+      </c>
+      <c r="E21" s="43" t="n">
+        <v>37500</v>
+      </c>
+      <c r="F21" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="G21" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J21" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="K21" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="10"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="41" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="41" t="s">
+        <v>104</v>
+      </c>
+      <c r="C22" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="D22" s="43" t="n">
+        <v>75</v>
+      </c>
+      <c r="E22" s="43" t="n">
+        <v>22500</v>
+      </c>
+      <c r="F22" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G22" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J22" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="K22" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="10"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="41" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="C23" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="D23" s="43" t="n">
+        <v>75</v>
+      </c>
+      <c r="E23" s="43" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F23" s="41" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J23" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="K23" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="10"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="41" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="41" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="42" t="n">
+        <v>100</v>
+      </c>
+      <c r="D24" s="43" t="n">
+        <v>550</v>
+      </c>
+      <c r="E24" s="43" t="n">
+        <v>55000</v>
+      </c>
+      <c r="F24" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G24" s="42" t="n">
+        <v>46</v>
+      </c>
+      <c r="H24" s="43" t="n">
+        <v>37922.88</v>
+      </c>
+      <c r="I24" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="J24" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K24" s="45" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="L24" s="45" t="n">
+        <v>0.689506909090909</v>
+      </c>
+      <c r="M24" s="10"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="41" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="41" t="s">
+        <v>64</v>
+      </c>
+      <c r="C25" s="42" t="n">
+        <v>100</v>
+      </c>
+      <c r="D25" s="43" t="n">
+        <v>550</v>
+      </c>
+      <c r="E25" s="43" t="n">
+        <v>55000</v>
+      </c>
+      <c r="F25" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G25" s="42" t="n">
+        <v>30</v>
+      </c>
+      <c r="H25" s="43" t="n">
+        <v>21838.24</v>
+      </c>
+      <c r="I25" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="J25" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K25" s="45" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L25" s="45" t="n">
+        <v>0.397058909090909</v>
+      </c>
+      <c r="M25" s="10"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="41" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" s="41" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="D26" s="43" t="n">
+        <v>265</v>
+      </c>
+      <c r="E26" s="43" t="n">
+        <v>53000</v>
+      </c>
+      <c r="F26" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G26" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J26" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="K26" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="10"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="41" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" s="41" t="s">
+        <v>67</v>
+      </c>
+      <c r="C27" s="42" t="n">
+        <v>50</v>
+      </c>
+      <c r="D27" s="43" t="n">
+        <v>350</v>
+      </c>
+      <c r="E27" s="43" t="n">
+        <v>17500</v>
+      </c>
+      <c r="F27" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G27" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J27" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="K27" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="10"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="41" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="41" t="s">
+        <v>68</v>
+      </c>
+      <c r="C28" s="42" t="n">
+        <v>60</v>
+      </c>
+      <c r="D28" s="43" t="n">
+        <v>440</v>
+      </c>
+      <c r="E28" s="43" t="n">
+        <v>26400</v>
+      </c>
+      <c r="F28" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G28" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J28" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="K28" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="10"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="41" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="41" t="s">
+        <v>69</v>
+      </c>
+      <c r="C29" s="42" t="n">
+        <v>350</v>
+      </c>
+      <c r="D29" s="43" t="n">
+        <v>160</v>
+      </c>
+      <c r="E29" s="43" t="n">
+        <v>56000</v>
+      </c>
+      <c r="F29" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="G29" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J29" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="K29" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="10"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="41" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="41" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="E30" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="47" t="s">
+        <v>98</v>
+      </c>
+      <c r="G30" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J30" s="48" t="s">
+        <v>99</v>
+      </c>
+      <c r="K30" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="L30" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="M30" s="10"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="41" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="41" t="s">
+        <v>72</v>
+      </c>
+      <c r="C31" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="E31" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="F31" s="47" t="s">
+        <v>98</v>
+      </c>
+      <c r="G31" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="J31" s="48" t="s">
+        <v>99</v>
+      </c>
+      <c r="K31" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="L31" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="M31" s="10"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="41" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" s="41" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="D32" s="43" t="n">
+        <v>65</v>
+      </c>
+      <c r="E32" s="43" t="n">
+        <v>19500</v>
+      </c>
+      <c r="F32" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="G32" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="H32" s="43" t="n">
+        <v>406.05</v>
+      </c>
+      <c r="I32" s="41" t="s">
+        <v>20</v>
+      </c>
+      <c r="J32" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K32" s="45" t="n">
+        <v>0.0233333333333333</v>
+      </c>
+      <c r="L32" s="45" t="n">
+        <v>0.0208230769230769</v>
+      </c>
+      <c r="M32" s="10"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="41" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" s="41" t="s">
+        <v>75</v>
+      </c>
+      <c r="C33" s="42" t="n">
+        <v>100</v>
+      </c>
+      <c r="D33" s="43" t="n">
+        <v>75</v>
+      </c>
+      <c r="E33" s="43" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F33" s="41" t="s">
+        <v>19</v>
+      </c>
+      <c r="G33" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="43" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I33" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="J33" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="K33" s="45" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="L33" s="45" t="n">
+        <v>5.33333333333333E-006</v>
+      </c>
+      <c r="M33" s="10" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="49"/>
+      <c r="B35" s="50" t="s">
+        <v>108</v>
+      </c>
+      <c r="C35" s="51" t="n">
+        <v>16380</v>
+      </c>
+      <c r="D35" s="49"/>
+      <c r="E35" s="52" t="n">
+        <v>1434906</v>
+      </c>
+      <c r="F35" s="49"/>
+      <c r="G35" s="51" t="n">
+        <v>8271</v>
+      </c>
+      <c r="H35" s="52" t="n">
+        <v>672404.4</v>
+      </c>
+      <c r="I35" s="49"/>
+      <c r="J35" s="49"/>
+      <c r="K35" s="49"/>
+      <c r="L35" s="53" t="n">
+        <v>0.468605190862677</v>
+      </c>
+      <c r="M35" s="49"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="49"/>
+      <c r="B36" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36" s="51" t="n">
+        <v>16380</v>
+      </c>
+      <c r="D36" s="49"/>
+      <c r="E36" s="52" t="n">
+        <v>1434906</v>
+      </c>
+      <c r="F36" s="49"/>
+      <c r="G36" s="51" t="n">
+        <v>8220</v>
+      </c>
+      <c r="H36" s="52" t="n">
+        <v>667610.16</v>
+      </c>
+      <c r="I36" s="49"/>
+      <c r="J36" s="49"/>
+      <c r="K36" s="53" t="n">
+        <v>0.501831501831502</v>
+      </c>
+      <c r="L36" s="53" t="n">
+        <v>0.465264038201806</v>
+      </c>
+      <c r="M36" s="49"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:L3"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>